<commit_message>
Add word "tålmodighed" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AB50"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4424,9 +4424,95 @@
         <v/>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>601db868-9010-4d2e-b3a5-c843d1248ecf</v>
+      </c>
+      <c r="B50" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C50" t="str">
+        <v>tålmodighed</v>
+      </c>
+      <c r="D50" t="str">
+        <v>tålmodighed</v>
+      </c>
+      <c r="E50" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F50" t="str">
+        <v>en</v>
+      </c>
+      <c r="G50" t="str">
+        <v>-en</v>
+      </c>
+      <c r="H50" t="str">
+        <v>[tʌlˈmoˀðiˌheðˀ]</v>
+      </c>
+      <c r="I50" t="str">
+        <v>https://static.ordnet.dk/mp3/12003/12003467_1.mp3</v>
+      </c>
+      <c r="J50" t="str">
+        <v>det at kunne finde sig i lang ventetid, forgæves anstrengelser eller andet besvær uden at miste besindelsen</v>
+      </c>
+      <c r="K50" t="str">
+        <v>patience</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Udenlandske leverandører skylder dansk erhvervsliv milliarder. Men vejen til kontrakterne kræver både tålmodighed, det rette netværk og et helt nyt tempo. Hos Mekoprint i Nordjylland har de fundet opskriften.</v>
+      </c>
+      <c r="M50" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N50" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O50" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=t%C3%A5lmodighed</v>
+      </c>
+      <c r="P50" t="str">
+        <v/>
+      </c>
+      <c r="Q50" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R50" t="str">
+        <v/>
+      </c>
+      <c r="S50" t="str">
+        <v/>
+      </c>
+      <c r="T50" t="str">
+        <v/>
+      </c>
+      <c r="U50" t="str">
+        <v/>
+      </c>
+      <c r="V50" t="str">
+        <v/>
+      </c>
+      <c r="W50" t="str">
+        <v/>
+      </c>
+      <c r="X50" t="str">
+        <v/>
+      </c>
+      <c r="Y50" t="str">
+        <v/>
+      </c>
+      <c r="Z50" t="str">
+        <v/>
+      </c>
+      <c r="AA50" t="str">
+        <v/>
+      </c>
+      <c r="AB50" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB50"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "opskriften" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB50"/>
+  <dimension ref="A1:AB51"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4510,9 +4510,95 @@
         <v/>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>95c373b6-cd45-4b2b-a5fc-b1a5c830f6c1</v>
+      </c>
+      <c r="B51" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C51" t="str">
+        <v>opskriften</v>
+      </c>
+      <c r="D51" t="str">
+        <v>opskrift</v>
+      </c>
+      <c r="E51" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F51" t="str">
+        <v>en</v>
+      </c>
+      <c r="G51" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037702_1.mp3</v>
+      </c>
+      <c r="J51" t="str">
+        <v>skriftlig anvisning på hvordan især en madret laves eller et håndarbejde udføres</v>
+      </c>
+      <c r="K51" t="str">
+        <v>The recipe</v>
+      </c>
+      <c r="L51" t="str">
+        <v>Udenlandske leverandører skylder dansk erhvervsliv milliarder. Men vejen til kontrakterne kræver både tålmodighed, det rette netværk og et helt nyt tempo. Hos Mekoprint i Nordjylland har de fundet opskriften.</v>
+      </c>
+      <c r="M51" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N51" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O51" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=opskriften</v>
+      </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
+      <c r="Q51" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R51" t="str">
+        <v/>
+      </c>
+      <c r="S51" t="str">
+        <v/>
+      </c>
+      <c r="T51" t="str">
+        <v/>
+      </c>
+      <c r="U51" t="str">
+        <v/>
+      </c>
+      <c r="V51" t="str">
+        <v/>
+      </c>
+      <c r="W51" t="str">
+        <v/>
+      </c>
+      <c r="X51" t="str">
+        <v/>
+      </c>
+      <c r="Y51" t="str">
+        <v/>
+      </c>
+      <c r="Z51" t="str">
+        <v/>
+      </c>
+      <c r="AA51" t="str">
+        <v/>
+      </c>
+      <c r="AB51" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB51"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ligne" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB51"/>
+  <dimension ref="A1:AB52"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4596,9 +4596,95 @@
         <v/>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>3b614dff-3752-4442-9fe6-07915e5dae63</v>
+      </c>
+      <c r="B52" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C52" t="str">
+        <v>ligne</v>
+      </c>
+      <c r="D52" t="str">
+        <v>ligne</v>
+      </c>
+      <c r="E52" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H52" t="str">
+        <v>[ˈliːnə]</v>
+      </c>
+      <c r="I52" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030458_1.mp3</v>
+      </c>
+      <c r="J52" t="str">
+        <v>have lighed med i udseende</v>
+      </c>
+      <c r="K52" t="str">
+        <v>resemble</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Det kunne ligne en krukke guld for enden af regnbuen.</v>
+      </c>
+      <c r="M52" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N52" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O52" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=ligne</v>
+      </c>
+      <c r="P52" t="str">
+        <v/>
+      </c>
+      <c r="Q52" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R52" t="str">
+        <v/>
+      </c>
+      <c r="S52" t="str">
+        <v/>
+      </c>
+      <c r="T52" t="str">
+        <v/>
+      </c>
+      <c r="U52" t="str">
+        <v/>
+      </c>
+      <c r="V52" t="str">
+        <v/>
+      </c>
+      <c r="W52" t="str">
+        <v/>
+      </c>
+      <c r="X52" t="str">
+        <v/>
+      </c>
+      <c r="Y52" t="str">
+        <v/>
+      </c>
+      <c r="Z52" t="str">
+        <v/>
+      </c>
+      <c r="AA52" t="str">
+        <v/>
+      </c>
+      <c r="AB52" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB52"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "enden" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB52"/>
+  <dimension ref="A1:AB53"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4682,9 +4682,95 @@
         <v/>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2e06480f-1b1d-4867-a446-d664d734efeb</v>
+      </c>
+      <c r="B53" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C53" t="str">
+        <v>enden</v>
+      </c>
+      <c r="D53" t="str">
+        <v>ende</v>
+      </c>
+      <c r="E53" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F53" t="str">
+        <v>en</v>
+      </c>
+      <c r="G53" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H53" t="str">
+        <v>[ˈεnə]</v>
+      </c>
+      <c r="I53" t="str">
+        <v>https://static.ordnet.dk/mp3/11011/11011289_1.mp3</v>
+      </c>
+      <c r="J53" t="str">
+        <v>hver af de to yderste dele af en aflang genstand, et aflangt område el.lign.</v>
+      </c>
+      <c r="K53" t="str">
+        <v>the end</v>
+      </c>
+      <c r="L53" t="str">
+        <v>Det kunne ligne en krukke guld for enden af regnbuen.</v>
+      </c>
+      <c r="M53" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N53" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O53" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=enden</v>
+      </c>
+      <c r="P53" t="str">
+        <v/>
+      </c>
+      <c r="Q53" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R53" t="str">
+        <v/>
+      </c>
+      <c r="S53" t="str">
+        <v/>
+      </c>
+      <c r="T53" t="str">
+        <v/>
+      </c>
+      <c r="U53" t="str">
+        <v/>
+      </c>
+      <c r="V53" t="str">
+        <v/>
+      </c>
+      <c r="W53" t="str">
+        <v/>
+      </c>
+      <c r="X53" t="str">
+        <v/>
+      </c>
+      <c r="Y53" t="str">
+        <v/>
+      </c>
+      <c r="Z53" t="str">
+        <v/>
+      </c>
+      <c r="AA53" t="str">
+        <v/>
+      </c>
+      <c r="AB53" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB53"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "regnbuen" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB53"/>
+  <dimension ref="A1:AB54"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4768,9 +4768,95 @@
         <v/>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>d3be5bfc-b32e-4c62-9d05-94453864a32e</v>
+      </c>
+      <c r="B54" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C54" t="str">
+        <v>regnbuen</v>
+      </c>
+      <c r="D54" t="str">
+        <v>regnbue</v>
+      </c>
+      <c r="E54" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F54" t="str">
+        <v>en</v>
+      </c>
+      <c r="G54" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H54" t="str">
+        <v>[ˈʁɑjnˌbuːə]</v>
+      </c>
+      <c r="I54" t="str">
+        <v>https://static.ordnet.dk/mp3/11042/11042546_1.mp3</v>
+      </c>
+      <c r="J54" t="str">
+        <v>bue af lys i forskellige farver der ofte kan ses på himlen når det regner og solen samtidig skinner</v>
+      </c>
+      <c r="K54" t="str">
+        <v>The rainbow</v>
+      </c>
+      <c r="L54" t="str">
+        <v>Det kunne ligne en krukke guld for enden af regnbuen.</v>
+      </c>
+      <c r="M54" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N54" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O54" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=regnbuen</v>
+      </c>
+      <c r="P54" t="str">
+        <v/>
+      </c>
+      <c r="Q54" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R54" t="str">
+        <v/>
+      </c>
+      <c r="S54" t="str">
+        <v/>
+      </c>
+      <c r="T54" t="str">
+        <v/>
+      </c>
+      <c r="U54" t="str">
+        <v/>
+      </c>
+      <c r="V54" t="str">
+        <v/>
+      </c>
+      <c r="W54" t="str">
+        <v/>
+      </c>
+      <c r="X54" t="str">
+        <v/>
+      </c>
+      <c r="Y54" t="str">
+        <v/>
+      </c>
+      <c r="Z54" t="str">
+        <v/>
+      </c>
+      <c r="AA54" t="str">
+        <v/>
+      </c>
+      <c r="AB54" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB54"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "krukke" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB54"/>
+  <dimension ref="A1:AB55"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4854,9 +4854,95 @@
         <v/>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>c3bf367a-78b3-4c58-b7e8-43ed7134bd0e</v>
+      </c>
+      <c r="B55" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C55" t="str">
+        <v>krukke</v>
+      </c>
+      <c r="D55" t="str">
+        <v>krukke</v>
+      </c>
+      <c r="E55" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F55" t="str">
+        <v>en</v>
+      </c>
+      <c r="G55" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H55" t="str">
+        <v>[ˈkʁɔgə]</v>
+      </c>
+      <c r="I55" t="str">
+        <v>https://static.ordnet.dk/mp3/11028/11028253_1.mp3</v>
+      </c>
+      <c r="J55" t="str">
+        <v>cylinderformet eller buet beholder (af ler, glas, porcelæn e.l.) med flad bund og en åbning foroven; kan være forsynet med låg og én eller to hanke bruges fx til opbevaring af (flydende) madvarer, krydderier eller løse genstande</v>
+      </c>
+      <c r="K55" t="str">
+        <v>jar</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Det kunne ligne en krukke guld for enden af regnbuen.</v>
+      </c>
+      <c r="M55" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N55" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O55" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=krukke</v>
+      </c>
+      <c r="P55" t="str">
+        <v/>
+      </c>
+      <c r="Q55" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R55" t="str">
+        <v/>
+      </c>
+      <c r="S55" t="str">
+        <v/>
+      </c>
+      <c r="T55" t="str">
+        <v/>
+      </c>
+      <c r="U55" t="str">
+        <v/>
+      </c>
+      <c r="V55" t="str">
+        <v/>
+      </c>
+      <c r="W55" t="str">
+        <v/>
+      </c>
+      <c r="X55" t="str">
+        <v/>
+      </c>
+      <c r="Y55" t="str">
+        <v/>
+      </c>
+      <c r="Z55" t="str">
+        <v/>
+      </c>
+      <c r="AA55" t="str">
+        <v/>
+      </c>
+      <c r="AB55" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB55"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update translation of "ligne" in Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB55"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4628,7 +4628,7 @@
         <v>have lighed med i udseende</v>
       </c>
       <c r="K52" t="str">
-        <v>resemble</v>
+        <v>resemble, look like</v>
       </c>
       <c r="L52" t="str">
         <v>Det kunne ligne en krukke guld for enden af regnbuen.</v>

</xml_diff>

<commit_message>
Add word "modkøbsaftaler" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB55"/>
+  <dimension ref="A1:AB56"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4940,9 +4940,95 @@
         <v/>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>de1cd672-21c6-45b1-9a0e-b036c9f76971</v>
+      </c>
+      <c r="B56" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C56" t="str">
+        <v>modkøbsaftaler</v>
+      </c>
+      <c r="D56" t="str">
+        <v>modkøbsaftale</v>
+      </c>
+      <c r="E56" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F56" t="str">
+        <v>en</v>
+      </c>
+      <c r="G56" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v>sammensat af modkøbs + aftale</v>
+      </c>
+      <c r="K56" t="str">
+        <v>Counter-purchase agreements</v>
+      </c>
+      <c r="L56" t="str">
+        <v>Hos Erhvervsstyrelsen er der nemlig en konto, der viser, at den danske forsvarsindustri i øjeblikket har 30,2 mia. kr. til gode hos udenlandske leverandører, også kendt som modkøbsaftaler.</v>
+      </c>
+      <c r="M56" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N56" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O56" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=modk%C3%B8bsaftaler</v>
+      </c>
+      <c r="P56" t="str">
+        <v/>
+      </c>
+      <c r="Q56" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R56" t="str">
+        <v/>
+      </c>
+      <c r="S56" t="str">
+        <v/>
+      </c>
+      <c r="T56" t="str">
+        <v/>
+      </c>
+      <c r="U56" t="str">
+        <v/>
+      </c>
+      <c r="V56" t="str">
+        <v/>
+      </c>
+      <c r="W56" t="str">
+        <v/>
+      </c>
+      <c r="X56" t="str">
+        <v/>
+      </c>
+      <c r="Y56" t="str">
+        <v/>
+      </c>
+      <c r="Z56" t="str">
+        <v/>
+      </c>
+      <c r="AA56" t="str">
+        <v/>
+      </c>
+      <c r="AB56" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB56"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "øjeblikket" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB56"/>
+  <dimension ref="A1:AB57"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5026,9 +5026,95 @@
         <v/>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>910f135d-ee86-4292-ac17-c8f94dd9f3e9</v>
+      </c>
+      <c r="B57" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C57" t="str">
+        <v>øjeblikket</v>
+      </c>
+      <c r="D57" t="str">
+        <v>øjeblik</v>
+      </c>
+      <c r="E57" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F57" t="str">
+        <v>et</v>
+      </c>
+      <c r="G57" t="str">
+        <v>-ket, -ke, -kene</v>
+      </c>
+      <c r="H57" t="str">
+        <v>[ˈʌjəˈbleg]</v>
+      </c>
+      <c r="I57" t="str">
+        <v>https://static.ordnet.dk/mp3/12008/12008204_1.mp3</v>
+      </c>
+      <c r="J57" t="str">
+        <v>meget kort tidsrum; tidspunkt</v>
+      </c>
+      <c r="K57" t="str">
+        <v>the moment</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Hos Erhvervsstyrelsen er der nemlig en konto, der viser, at den danske forsvarsindustri i øjeblikket har 30,2 mia. kr. til gode hos udenlandske leverandører, også kendt som modkøbsaftaler.</v>
+      </c>
+      <c r="M57" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N57" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O57" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=%C3%B8jeblikket</v>
+      </c>
+      <c r="P57" t="str">
+        <v/>
+      </c>
+      <c r="Q57" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R57" t="str">
+        <v/>
+      </c>
+      <c r="S57" t="str">
+        <v/>
+      </c>
+      <c r="T57" t="str">
+        <v/>
+      </c>
+      <c r="U57" t="str">
+        <v/>
+      </c>
+      <c r="V57" t="str">
+        <v/>
+      </c>
+      <c r="W57" t="str">
+        <v/>
+      </c>
+      <c r="X57" t="str">
+        <v/>
+      </c>
+      <c r="Y57" t="str">
+        <v/>
+      </c>
+      <c r="Z57" t="str">
+        <v/>
+      </c>
+      <c r="AA57" t="str">
+        <v/>
+      </c>
+      <c r="AB57" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB57"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Kammer" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB57"/>
+  <dimension ref="A1:AB58"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5112,9 +5112,95 @@
         <v/>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>bf5f1ac6-b96a-4072-bbb4-207bac9a92a7</v>
+      </c>
+      <c r="B58" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Kammer</v>
+      </c>
+      <c r="D58" t="str">
+        <v>kammer</v>
+      </c>
+      <c r="E58" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F58" t="str">
+        <v>et</v>
+      </c>
+      <c r="G58" t="str">
+        <v>-et eller (uofficielt) kamret, kamre, kamrene</v>
+      </c>
+      <c r="H58" t="str">
+        <v>[ˈkɑmˀʌ]</v>
+      </c>
+      <c r="I58" t="str">
+        <v>https://static.ordnet.dk/mp3/11025/11025117_1.mp3</v>
+      </c>
+      <c r="J58" t="str">
+        <v>lille værelse</v>
+      </c>
+      <c r="K58" t="str">
+        <v>Chamber</v>
+      </c>
+      <c r="L58" t="str">
+        <v>Eller som Kammeradvokaten Poul Schmith skriver, skylder udenlandske leverandører lige nu dansk erhvervsliv 30,2 mia. kr. i modkøb, som de skal afvikle inden for få år.</v>
+      </c>
+      <c r="M58" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N58" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O58" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=Kammer</v>
+      </c>
+      <c r="P58" t="str">
+        <v/>
+      </c>
+      <c r="Q58" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R58" t="str">
+        <v/>
+      </c>
+      <c r="S58" t="str">
+        <v/>
+      </c>
+      <c r="T58" t="str">
+        <v/>
+      </c>
+      <c r="U58" t="str">
+        <v/>
+      </c>
+      <c r="V58" t="str">
+        <v/>
+      </c>
+      <c r="W58" t="str">
+        <v/>
+      </c>
+      <c r="X58" t="str">
+        <v/>
+      </c>
+      <c r="Y58" t="str">
+        <v/>
+      </c>
+      <c r="Z58" t="str">
+        <v/>
+      </c>
+      <c r="AA58" t="str">
+        <v/>
+      </c>
+      <c r="AB58" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB58"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "legendariske" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB58"/>
+  <dimension ref="A1:AB59"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5198,9 +5198,95 @@
         <v/>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>a164a6b6-c242-4681-85ed-cbe8c064a132</v>
+      </c>
+      <c r="B59" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C59" t="str">
+        <v>legendariske</v>
+      </c>
+      <c r="D59" t="str">
+        <v>legendarisk</v>
+      </c>
+      <c r="E59" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+      <c r="G59" t="str">
+        <v>-, -e</v>
+      </c>
+      <c r="H59" t="str">
+        <v>[legənˈdɑˀisg]</v>
+      </c>
+      <c r="I59" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030082_1.mp3</v>
+      </c>
+      <c r="J59" t="str">
+        <v>som hører til, minder om eller findes i legender</v>
+      </c>
+      <c r="K59" t="str">
+        <v>Legendary</v>
+      </c>
+      <c r="L59" t="str">
+        <v>Siden december 2025 er det tal bare steget og steget, hvilket følger i kølvandet på statsminister Mette Frederiksens nu legendariske opfordring til den danske forsvarschef i februar 2025: “Køb, køb, køb”.</v>
+      </c>
+      <c r="M59" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N59" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O59" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=legendariske</v>
+      </c>
+      <c r="P59" t="str">
+        <v/>
+      </c>
+      <c r="Q59" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R59" t="str">
+        <v/>
+      </c>
+      <c r="S59" t="str">
+        <v/>
+      </c>
+      <c r="T59" t="str">
+        <v/>
+      </c>
+      <c r="U59" t="str">
+        <v/>
+      </c>
+      <c r="V59" t="str">
+        <v/>
+      </c>
+      <c r="W59" t="str">
+        <v/>
+      </c>
+      <c r="X59" t="str">
+        <v/>
+      </c>
+      <c r="Y59" t="str">
+        <v/>
+      </c>
+      <c r="Z59" t="str">
+        <v/>
+      </c>
+      <c r="AA59" t="str">
+        <v/>
+      </c>
+      <c r="AB59" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB59"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "opfordring" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB59"/>
+  <dimension ref="A1:AB60"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5284,9 +5284,95 @@
         <v/>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>ad82d9aa-44db-485e-b296-186579372488</v>
+      </c>
+      <c r="B60" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C60" t="str">
+        <v>opfordring</v>
+      </c>
+      <c r="D60" t="str">
+        <v>opfordring</v>
+      </c>
+      <c r="E60" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F60" t="str">
+        <v>en</v>
+      </c>
+      <c r="G60" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H60" t="str">
+        <v>[-ˌfɒˀdʁεŋ]</v>
+      </c>
+      <c r="I60" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037419_1.mp3</v>
+      </c>
+      <c r="J60" t="str">
+        <v>det at opfordre nogen til noget; ytring der opfordrer nogen til noget</v>
+      </c>
+      <c r="K60" t="str">
+        <v>Request</v>
+      </c>
+      <c r="L60" t="str">
+        <v>Siden december 2025 er det tal bare steget og steget, hvilket følger i kølvandet på statsminister Mette Frederiksens nu legendariske opfordring til den danske forsvarschef i februar 2025: “Køb, køb, køb”.</v>
+      </c>
+      <c r="M60" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N60" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O60" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=opfordring</v>
+      </c>
+      <c r="P60" t="str">
+        <v/>
+      </c>
+      <c r="Q60" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R60" t="str">
+        <v/>
+      </c>
+      <c r="S60" t="str">
+        <v/>
+      </c>
+      <c r="T60" t="str">
+        <v/>
+      </c>
+      <c r="U60" t="str">
+        <v/>
+      </c>
+      <c r="V60" t="str">
+        <v/>
+      </c>
+      <c r="W60" t="str">
+        <v/>
+      </c>
+      <c r="X60" t="str">
+        <v/>
+      </c>
+      <c r="Y60" t="str">
+        <v/>
+      </c>
+      <c r="Z60" t="str">
+        <v/>
+      </c>
+      <c r="AA60" t="str">
+        <v/>
+      </c>
+      <c r="AB60" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB60"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "i kø" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB60"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5379,30 +5379,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5813,9 +5813,77 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>27d9bc7f-1ef2-41f3-9566-24aad6f7bac6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C7" t="str">
+        <v>i kø</v>
+      </c>
+      <c r="D7" t="str">
+        <v>i=in · kø=queue</v>
+      </c>
+      <c r="E7" t="str">
+        <v>in queue</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Og nu står modkøbsaftalerne i kø på Erhversstyrelsens hjemmeside. Det gælder for eksempel britiske BAE Systems Hägglunds der er forpligtet til at købe for over fire milliarder kroner hos danske virksomheder fordi de blandt andet skal levere 44 CV90 infanterikampkøretøjer. Eller den norske missilproducent Kongsberg Defence &amp; Aerospace AS, der skal købe for over fem milliarder kroner for levering af forskellige missilsystemer.</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="H7" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=i%20k%C3%B8</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "gælder" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB60"/>
+  <dimension ref="A1:AB61"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5370,9 +5370,95 @@
         <v/>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>01004d86-e2d2-4c06-b23d-6918a651b20d</v>
+      </c>
+      <c r="B61" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C61" t="str">
+        <v>gælder</v>
+      </c>
+      <c r="D61" t="str">
+        <v>gælde</v>
+      </c>
+      <c r="E61" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v>-r, gjaldt, gjaldt (eller gældt)</v>
+      </c>
+      <c r="H61" t="str">
+        <v>[ˈgεlə]</v>
+      </c>
+      <c r="I61" t="str">
+        <v>https://static.ordnet.dk/mp3/11019/11019346_1.mp3</v>
+      </c>
+      <c r="J61" t="str">
+        <v>være gyldig; have gyldighed</v>
+      </c>
+      <c r="K61" t="str">
+        <v>applies</v>
+      </c>
+      <c r="L61" t="str">
+        <v>Og nu står modkøbsaftalerne i kø på Erhversstyrelsens hjemmeside. Det gælder for eksempel britiske BAE Systems Hägglunds der er forpligtet til at købe for over fire milliarder kroner hos danske virksomheder fordi de blandt andet skal levere 44 CV90 infanterikampkøretøjer. Eller den norske missilproducent Kongsberg Defence &amp; Aerospace AS, der skal købe for over fem milliarder kroner for levering af forskellige missilsystemer.</v>
+      </c>
+      <c r="M61" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N61" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O61" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=g%C3%A6lder</v>
+      </c>
+      <c r="P61" t="str">
+        <v/>
+      </c>
+      <c r="Q61" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R61" t="str">
+        <v/>
+      </c>
+      <c r="S61" t="str">
+        <v/>
+      </c>
+      <c r="T61" t="str">
+        <v/>
+      </c>
+      <c r="U61" t="str">
+        <v/>
+      </c>
+      <c r="V61" t="str">
+        <v/>
+      </c>
+      <c r="W61" t="str">
+        <v/>
+      </c>
+      <c r="X61" t="str">
+        <v/>
+      </c>
+      <c r="Y61" t="str">
+        <v/>
+      </c>
+      <c r="Z61" t="str">
+        <v/>
+      </c>
+      <c r="AA61" t="str">
+        <v/>
+      </c>
+      <c r="AB61" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5381,28 +5467,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V7"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "forpligtet" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB61"/>
+  <dimension ref="A1:AB62"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5456,9 +5456,95 @@
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>6ecd1790-b66f-4e0c-9e77-da387e4dbee1</v>
+      </c>
+      <c r="B62" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C62" t="str">
+        <v>forpligtet</v>
+      </c>
+      <c r="D62" t="str">
+        <v>forpligte</v>
+      </c>
+      <c r="E62" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H62" t="str">
+        <v>[fʌˈplegdə]</v>
+      </c>
+      <c r="I62" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014958_1.mp3</v>
+      </c>
+      <c r="J62" t="str">
+        <v>gøre bundet af en lov, en (uskreven eller moralsk) regel, et løfte el.lign.</v>
+      </c>
+      <c r="K62" t="str">
+        <v>obliged</v>
+      </c>
+      <c r="L62" t="str">
+        <v>Og nu står modkøbsaftalerne i kø på Erhversstyrelsens hjemmeside. Det gælder for eksempel britiske BAE Systems Hägglunds der er forpligtet til at købe for over fire milliarder kroner hos danske virksomheder fordi de blandt andet skal levere 44 CV90 infanterikampkøretøjer. Eller den norske missilproducent Kongsberg Defence &amp; Aerospace AS, der skal købe for over fem milliarder kroner for levering af forskellige missilsystemer.</v>
+      </c>
+      <c r="M62" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N62" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O62" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=forpligtet</v>
+      </c>
+      <c r="P62" t="str">
+        <v/>
+      </c>
+      <c r="Q62" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R62" t="str">
+        <v/>
+      </c>
+      <c r="S62" t="str">
+        <v/>
+      </c>
+      <c r="T62" t="str">
+        <v/>
+      </c>
+      <c r="U62" t="str">
+        <v/>
+      </c>
+      <c r="V62" t="str">
+        <v/>
+      </c>
+      <c r="W62" t="str">
+        <v/>
+      </c>
+      <c r="X62" t="str">
+        <v/>
+      </c>
+      <c r="Y62" t="str">
+        <v/>
+      </c>
+      <c r="Z62" t="str">
+        <v/>
+      </c>
+      <c r="AA62" t="str">
+        <v/>
+      </c>
+      <c r="AB62" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB62"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ethvert" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB62"/>
+  <dimension ref="A1:AB63"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5542,9 +5542,95 @@
         <v/>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>efb26386-aad7-45e3-8e5d-9164aea1db5c</v>
+      </c>
+      <c r="B63" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C63" t="str">
+        <v>ethvert</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v>pronomen</v>
+      </c>
+      <c r="F63" t="str">
+        <v>et</v>
+      </c>
+      <c r="G63" t="str">
+        <v>intetkøn: ethvert</v>
+      </c>
+      <c r="H63" t="str">
+        <v>[enˈvεɐ̯ˀ]</v>
+      </c>
+      <c r="I63" t="str">
+        <v>https://static.ordnet.dk/mp3/11011/11011446_1.mp3</v>
+      </c>
+      <c r="J63" t="str">
+        <v>hver enkelt person eller ting i en helhed uden undtagelse</v>
+      </c>
+      <c r="K63" t="str">
+        <v>Any</v>
+      </c>
+      <c r="L63" t="str">
+        <v>Men som i ethvert eventyr er de mange penge ikke så nemme at få fat i, hvis man er den nye i klassen. Det kræver både tålmodighed og et godt netværk, lyder det fra to af Danmarks største erhvervsorganisationer.</v>
+      </c>
+      <c r="M63" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N63" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O63" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=ethvert</v>
+      </c>
+      <c r="P63" t="str">
+        <v/>
+      </c>
+      <c r="Q63" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R63" t="str">
+        <v/>
+      </c>
+      <c r="S63" t="str">
+        <v/>
+      </c>
+      <c r="T63" t="str">
+        <v/>
+      </c>
+      <c r="U63" t="str">
+        <v/>
+      </c>
+      <c r="V63" t="str">
+        <v/>
+      </c>
+      <c r="W63" t="str">
+        <v/>
+      </c>
+      <c r="X63" t="str">
+        <v/>
+      </c>
+      <c r="Y63" t="str">
+        <v/>
+      </c>
+      <c r="Z63" t="str">
+        <v/>
+      </c>
+      <c r="AA63" t="str">
+        <v/>
+      </c>
+      <c r="AB63" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "at få fat i" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB63"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5637,30 +5637,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V8"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6139,9 +6139,77 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>e5878213-c794-4ab8-880a-c5bb5dd2f84e</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C8" t="str">
+        <v>at få fat i</v>
+      </c>
+      <c r="D8" t="str">
+        <v>at=to · få=get · fat=Fat · i=in</v>
+      </c>
+      <c r="E8" t="str">
+        <v>to get hold of</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Men som i ethvert eventyr er de mange penge ikke så nemme at få fat i, hvis man er den nye i klassen. Det kræver både tålmodighed og et godt netværk, lyder det fra to af Danmarks største erhvervsorganisationer.</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="H8" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=at%20f%C3%A5%20fat%20i</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "vendt på hovedet" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -5637,7 +5637,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6207,9 +6207,77 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>6f3a1dee-4bee-41ae-91d1-6588a01c5220</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C9" t="str">
+        <v>vendt på hovedet</v>
+      </c>
+      <c r="D9" t="str">
+        <v>vendt=turned · på=on · hovedet=the head</v>
+      </c>
+      <c r="E9" t="str">
+        <v>turned upside down</v>
+      </c>
+      <c r="F9" t="str">
+        <v>»Hvor pris og kvalitet tidligere har været de vigtigste faktorer, så er det nu vendt på hovedet, og hastighed er i dag helt afgørende. Det giver plads til nye virksomheder,« siger Joachim Finkielman, der er direktør i DI Forsvar og Sikkerhed.</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="H9" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=vendt%20p%C3%A5%20hovedet</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "hastighed" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB63"/>
+  <dimension ref="A1:AB64"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5628,9 +5628,95 @@
         <v/>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>8c60630c-0b46-42ae-9586-360994fd4104</v>
+      </c>
+      <c r="B64" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C64" t="str">
+        <v>hastighed</v>
+      </c>
+      <c r="D64" t="str">
+        <v>hastighed</v>
+      </c>
+      <c r="E64" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F64" t="str">
+        <v>en</v>
+      </c>
+      <c r="G64" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H64" t="str">
+        <v>[ˈhasdiˌheðˀ]</v>
+      </c>
+      <c r="I64" t="str">
+        <v>https://static.ordnet.dk/mp3/11019/11019997_1.mp3</v>
+      </c>
+      <c r="J64" t="str">
+        <v>den hurtighed eller fart som noget foregår eller bevæger sig med, ofte udtrykt som forholdet mellem tilbagelagt strækning og anvendt tid</v>
+      </c>
+      <c r="K64" t="str">
+        <v>speed</v>
+      </c>
+      <c r="L64" t="str">
+        <v>»Hvor pris og kvalitet tidligere har været de vigtigste faktorer, så er det nu vendt på hovedet, og hastighed er i dag helt afgørende. Det giver plads til nye virksomheder,« siger Joachim Finkielman, der er direktør i DI Forsvar og Sikkerhed.</v>
+      </c>
+      <c r="M64" t="str">
+        <v>Pengene sidder løst i Forsvaret: Sådan får danske tech-virksomheder del i »køb, køb, køb« | Ingeniøren</v>
+      </c>
+      <c r="N64" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb</v>
+      </c>
+      <c r="O64" t="str">
+        <v>https://ing.dk/artikel/pengene-sidder-loest-i-forsvaret-saadan-faar-danske-tech-virksomheder-del-i-koeb-koeb-koeb#:~:text=hastighed</v>
+      </c>
+      <c r="P64" t="str">
+        <v/>
+      </c>
+      <c r="Q64" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R64" t="str">
+        <v/>
+      </c>
+      <c r="S64" t="str">
+        <v/>
+      </c>
+      <c r="T64" t="str">
+        <v/>
+      </c>
+      <c r="U64" t="str">
+        <v/>
+      </c>
+      <c r="V64" t="str">
+        <v/>
+      </c>
+      <c r="W64" t="str">
+        <v/>
+      </c>
+      <c r="X64" t="str">
+        <v/>
+      </c>
+      <c r="Y64" t="str">
+        <v/>
+      </c>
+      <c r="Z64" t="str">
+        <v/>
+      </c>
+      <c r="AA64" t="str">
+        <v/>
+      </c>
+      <c r="AB64" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB64"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5639,28 +5725,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V9"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "lovet" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB64"/>
+  <dimension ref="A1:AB65"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5714,9 +5714,95 @@
         <v/>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>c4d0f4b2-91e4-4a0c-855c-14c31eb898ab</v>
+      </c>
+      <c r="B65" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C65" t="str">
+        <v>lovet</v>
+      </c>
+      <c r="D65" t="str">
+        <v>love</v>
+      </c>
+      <c r="E65" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+      <c r="G65" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H65" t="str">
+        <v>[ˈlɔːwə]</v>
+      </c>
+      <c r="I65" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030997_1.mp3</v>
+      </c>
+      <c r="J65" t="str">
+        <v>give nogen et løfte</v>
+      </c>
+      <c r="K65" t="str">
+        <v>promised</v>
+      </c>
+      <c r="L65" t="str">
+        <v>Novo-ledelsen har lovet at blive både hurtigere og bedre til at udvikle ny medicin, og her er kunstig intelligens en hjørnesten til at bygge det nye Novo.</v>
+      </c>
+      <c r="M65" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N65" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O65" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=lovet</v>
+      </c>
+      <c r="P65" t="str">
+        <v/>
+      </c>
+      <c r="Q65" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R65" t="str">
+        <v/>
+      </c>
+      <c r="S65" t="str">
+        <v/>
+      </c>
+      <c r="T65" t="str">
+        <v/>
+      </c>
+      <c r="U65" t="str">
+        <v/>
+      </c>
+      <c r="V65" t="str">
+        <v/>
+      </c>
+      <c r="W65" t="str">
+        <v/>
+      </c>
+      <c r="X65" t="str">
+        <v/>
+      </c>
+      <c r="Y65" t="str">
+        <v/>
+      </c>
+      <c r="Z65" t="str">
+        <v/>
+      </c>
+      <c r="AA65" t="str">
+        <v/>
+      </c>
+      <c r="AB65" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB65"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kunstig" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB65"/>
+  <dimension ref="A1:AB66"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5800,9 +5800,95 @@
         <v/>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>993562f3-46a1-4304-8788-ccda2cefd125</v>
+      </c>
+      <c r="B66" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C66" t="str">
+        <v>kunstig</v>
+      </c>
+      <c r="D66" t="str">
+        <v>kunstig</v>
+      </c>
+      <c r="E66" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+      <c r="G66" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H66" t="str">
+        <v>[ˈkɔnsdi]</v>
+      </c>
+      <c r="I66" t="str">
+        <v>https://static.ordnet.dk/mp3/11028/11028635_1.mp3</v>
+      </c>
+      <c r="J66" t="str">
+        <v>frembragt eller arrangeret af mennesker som en efterligning af noget der ellers forekommer i naturen eller sker naturligt</v>
+      </c>
+      <c r="K66" t="str">
+        <v>artificial</v>
+      </c>
+      <c r="L66" t="str">
+        <v>Novo-ledelsen har lovet at blive både hurtigere og bedre til at udvikle ny medicin, og her er kunstig intelligens en hjørnesten til at bygge det nye Novo.</v>
+      </c>
+      <c r="M66" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N66" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O66" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=kunstig</v>
+      </c>
+      <c r="P66" t="str">
+        <v/>
+      </c>
+      <c r="Q66" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R66" t="str">
+        <v/>
+      </c>
+      <c r="S66" t="str">
+        <v/>
+      </c>
+      <c r="T66" t="str">
+        <v/>
+      </c>
+      <c r="U66" t="str">
+        <v/>
+      </c>
+      <c r="V66" t="str">
+        <v/>
+      </c>
+      <c r="W66" t="str">
+        <v/>
+      </c>
+      <c r="X66" t="str">
+        <v/>
+      </c>
+      <c r="Y66" t="str">
+        <v/>
+      </c>
+      <c r="Z66" t="str">
+        <v/>
+      </c>
+      <c r="AA66" t="str">
+        <v/>
+      </c>
+      <c r="AB66" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB66"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "hjørnesten" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB66"/>
+  <dimension ref="A1:AB67"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5886,9 +5886,95 @@
         <v/>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>14722365-4f3b-44e4-b0a6-1d5973f405d5</v>
+      </c>
+      <c r="B67" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C67" t="str">
+        <v>hjørnesten</v>
+      </c>
+      <c r="D67" t="str">
+        <v>hjørnesten</v>
+      </c>
+      <c r="E67" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F67" t="str">
+        <v>en</v>
+      </c>
+      <c r="G67" t="str">
+        <v>-en, - eller -e, -ene Se bøjning i skema</v>
+      </c>
+      <c r="H67" t="str">
+        <v/>
+      </c>
+      <c r="I67" t="str">
+        <v>https://static.ordnet.dk/mp3/11021/11021112_1.mp3</v>
+      </c>
+      <c r="J67" t="str">
+        <v>grundsten under et hjørne af et hus</v>
+      </c>
+      <c r="K67" t="str">
+        <v>Cornerstone</v>
+      </c>
+      <c r="L67" t="str">
+        <v>Novo-ledelsen har lovet at blive både hurtigere og bedre til at udvikle ny medicin, og her er kunstig intelligens en hjørnesten til at bygge det nye Novo.</v>
+      </c>
+      <c r="M67" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N67" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O67" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=hj%C3%B8rnesten</v>
+      </c>
+      <c r="P67" t="str">
+        <v/>
+      </c>
+      <c r="Q67" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R67" t="str">
+        <v/>
+      </c>
+      <c r="S67" t="str">
+        <v/>
+      </c>
+      <c r="T67" t="str">
+        <v/>
+      </c>
+      <c r="U67" t="str">
+        <v/>
+      </c>
+      <c r="V67" t="str">
+        <v/>
+      </c>
+      <c r="W67" t="str">
+        <v/>
+      </c>
+      <c r="X67" t="str">
+        <v/>
+      </c>
+      <c r="Y67" t="str">
+        <v/>
+      </c>
+      <c r="Z67" t="str">
+        <v/>
+      </c>
+      <c r="AA67" t="str">
+        <v/>
+      </c>
+      <c r="AB67" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB67"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "nærmest" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB67"/>
+  <dimension ref="A1:AB68"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5972,9 +5972,95 @@
         <v/>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>133b713a-0b11-4727-bf5a-bd1c4a34f0dd</v>
+      </c>
+      <c r="B68" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C68" t="str">
+        <v>nærmest</v>
+      </c>
+      <c r="D68" t="str">
+        <v>nærmest</v>
+      </c>
+      <c r="E68" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+      <c r="G68" t="str">
+        <v>-, -e, som prædikativ: -</v>
+      </c>
+      <c r="H68" t="str">
+        <v>[ˈnæɐ̯məsd]</v>
+      </c>
+      <c r="I68" t="str">
+        <v>https://static.ordnet.dk/mp3/11036/11036538_1.mp3</v>
+      </c>
+      <c r="J68" t="str">
+        <v>superlativ af nær</v>
+      </c>
+      <c r="K68" t="str">
+        <v>closest</v>
+      </c>
+      <c r="L68" t="str">
+        <v>Mike Doustdar vil have sine ansatte til at være dedikerede - nærmest besatte - i jagten på fremtidens guld, og med tidens største mestre inden for computerhjerner vælger topchefen AI-værktøjskassen som sit våben over for Novos skarpladte konkurrenter.</v>
+      </c>
+      <c r="M68" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N68" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O68" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=n%C3%A6rmest</v>
+      </c>
+      <c r="P68" t="str">
+        <v/>
+      </c>
+      <c r="Q68" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R68" t="str">
+        <v/>
+      </c>
+      <c r="S68" t="str">
+        <v/>
+      </c>
+      <c r="T68" t="str">
+        <v/>
+      </c>
+      <c r="U68" t="str">
+        <v/>
+      </c>
+      <c r="V68" t="str">
+        <v/>
+      </c>
+      <c r="W68" t="str">
+        <v/>
+      </c>
+      <c r="X68" t="str">
+        <v/>
+      </c>
+      <c r="Y68" t="str">
+        <v/>
+      </c>
+      <c r="Z68" t="str">
+        <v/>
+      </c>
+      <c r="AA68" t="str">
+        <v/>
+      </c>
+      <c r="AB68" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB68"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "dedikerede" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB68"/>
+  <dimension ref="A1:AB69"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6058,9 +6058,95 @@
         <v/>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>617a0721-8721-4abe-bd9d-cef59b972248</v>
+      </c>
+      <c r="B69" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C69" t="str">
+        <v>dedikerede</v>
+      </c>
+      <c r="D69" t="str">
+        <v>dedicere</v>
+      </c>
+      <c r="E69" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+      <c r="G69" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H69" t="str">
+        <v>[dediˈseˀʌ]</v>
+      </c>
+      <c r="I69" t="str">
+        <v>https://static.ordnet.dk/mp3/11008/11008537_1.mp3</v>
+      </c>
+      <c r="J69" t="str">
+        <v>tilegne (en bog, sang e.l.) til nogen som tegn på agtelse eller varme følelser</v>
+      </c>
+      <c r="K69" t="str">
+        <v>Dedicated</v>
+      </c>
+      <c r="L69" t="str">
+        <v>Mike Doustdar vil have sine ansatte til at være dedikerede - nærmest besatte - i jagten på fremtidens guld, og med tidens største mestre inden for computerhjerner vælger topchefen AI-værktøjskassen som sit våben over for Novos skarpladte konkurrenter.</v>
+      </c>
+      <c r="M69" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N69" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O69" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=dedikerede</v>
+      </c>
+      <c r="P69" t="str">
+        <v/>
+      </c>
+      <c r="Q69" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R69" t="str">
+        <v/>
+      </c>
+      <c r="S69" t="str">
+        <v/>
+      </c>
+      <c r="T69" t="str">
+        <v/>
+      </c>
+      <c r="U69" t="str">
+        <v/>
+      </c>
+      <c r="V69" t="str">
+        <v/>
+      </c>
+      <c r="W69" t="str">
+        <v/>
+      </c>
+      <c r="X69" t="str">
+        <v/>
+      </c>
+      <c r="Y69" t="str">
+        <v/>
+      </c>
+      <c r="Z69" t="str">
+        <v/>
+      </c>
+      <c r="AA69" t="str">
+        <v/>
+      </c>
+      <c r="AB69" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB69"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "besatte" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB69"/>
+  <dimension ref="A1:AB70"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6144,9 +6144,95 @@
         <v/>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>7392d09d-da98-4183-91f7-c150de1b473c</v>
+      </c>
+      <c r="B70" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C70" t="str">
+        <v>besatte</v>
+      </c>
+      <c r="D70" t="str">
+        <v>besætte</v>
+      </c>
+      <c r="E70" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+      <c r="G70" t="str">
+        <v>-r, besatte, besat</v>
+      </c>
+      <c r="H70" t="str">
+        <v>[beˈsεdə]</v>
+      </c>
+      <c r="I70" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004371_1.mp3</v>
+      </c>
+      <c r="J70" t="str">
+        <v>indtage og derefter kontrollere et land, et landområde el.lign. ved militær magtanvendelse</v>
+      </c>
+      <c r="K70" t="str">
+        <v>occupied</v>
+      </c>
+      <c r="L70" t="str">
+        <v>Mike Doustdar vil have sine ansatte til at være dedikerede - nærmest besatte - i jagten på fremtidens guld, og med tidens største mestre inden for computerhjerner vælger topchefen AI-værktøjskassen som sit våben over for Novos skarpladte konkurrenter.</v>
+      </c>
+      <c r="M70" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N70" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O70" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=besatte</v>
+      </c>
+      <c r="P70" t="str">
+        <v/>
+      </c>
+      <c r="Q70" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R70" t="str">
+        <v/>
+      </c>
+      <c r="S70" t="str">
+        <v/>
+      </c>
+      <c r="T70" t="str">
+        <v/>
+      </c>
+      <c r="U70" t="str">
+        <v/>
+      </c>
+      <c r="V70" t="str">
+        <v/>
+      </c>
+      <c r="W70" t="str">
+        <v/>
+      </c>
+      <c r="X70" t="str">
+        <v/>
+      </c>
+      <c r="Y70" t="str">
+        <v/>
+      </c>
+      <c r="Z70" t="str">
+        <v/>
+      </c>
+      <c r="AA70" t="str">
+        <v/>
+      </c>
+      <c r="AB70" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB70"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "mestre" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB70"/>
+  <dimension ref="A1:AB71"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6230,9 +6230,95 @@
         <v/>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>2bb19328-ec31-422b-9a44-b415feee8221</v>
+      </c>
+      <c r="B71" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C71" t="str">
+        <v>mestre</v>
+      </c>
+      <c r="D71" t="str">
+        <v>mestre</v>
+      </c>
+      <c r="E71" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H71" t="str">
+        <v>[ˈmεsdʁʌ]</v>
+      </c>
+      <c r="I71" t="str">
+        <v>https://static.ordnet.dk/mp3/11033/11033333_1.mp3</v>
+      </c>
+      <c r="J71" t="str">
+        <v>klare, håndtere eller beherske noget vanskeligt, svært eller kompliceret uden problemer</v>
+      </c>
+      <c r="K71" t="str">
+        <v>master</v>
+      </c>
+      <c r="L71" t="str">
+        <v>Mike Doustdar vil have sine ansatte til at være dedikerede - nærmest besatte - i jagten på fremtidens guld, og med tidens største mestre inden for computerhjerner vælger topchefen AI-værktøjskassen som sit våben over for Novos skarpladte konkurrenter.</v>
+      </c>
+      <c r="M71" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N71" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O71" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=mestre</v>
+      </c>
+      <c r="P71" t="str">
+        <v/>
+      </c>
+      <c r="Q71" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R71" t="str">
+        <v/>
+      </c>
+      <c r="S71" t="str">
+        <v/>
+      </c>
+      <c r="T71" t="str">
+        <v/>
+      </c>
+      <c r="U71" t="str">
+        <v/>
+      </c>
+      <c r="V71" t="str">
+        <v/>
+      </c>
+      <c r="W71" t="str">
+        <v/>
+      </c>
+      <c r="X71" t="str">
+        <v/>
+      </c>
+      <c r="Y71" t="str">
+        <v/>
+      </c>
+      <c r="Z71" t="str">
+        <v/>
+      </c>
+      <c r="AA71" t="str">
+        <v/>
+      </c>
+      <c r="AB71" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB71"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "udvekslings" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB71"/>
+  <dimension ref="A1:AB72"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6316,9 +6316,95 @@
         <v/>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>9e980f2b-cde2-4d06-af77-83ffb9c991ed</v>
+      </c>
+      <c r="B72" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C72" t="str">
+        <v>udvekslings</v>
+      </c>
+      <c r="D72" t="str">
+        <v>udveksling</v>
+      </c>
+      <c r="E72" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F72" t="str">
+        <v>en</v>
+      </c>
+      <c r="G72" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H72" t="str">
+        <v/>
+      </c>
+      <c r="I72" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004281_1.mp3</v>
+      </c>
+      <c r="J72" t="str">
+        <v>det at give noget i bytte for noget andet, som regel af samme slags</v>
+      </c>
+      <c r="K72" t="str">
+        <v>Exchange</v>
+      </c>
+      <c r="L72" t="str">
+        <v>Kære studerende Drømmer du om at studere i udlandet som en del af din uddannelse? Den 1. november 2026 er ansøgningsfristen i efterårsrunden for udvekslingsophold i studieåret 2027/2028. For at hjælpe dig med at komme godt i gang holder International Office en række informationsmøder, hvor du kan høre mere om dine muligheder, ansøgnin …</v>
+      </c>
+      <c r="M72" t="str">
+        <v>Lecture 2 - Statistical Signal Processing, (E26) - itslearning</v>
+      </c>
+      <c r="N72" t="str">
+        <v>https://sdu.itslearning.com/plans/courses/50426/plan/407433?BackDestination=1</v>
+      </c>
+      <c r="O72" t="str">
+        <v>https://sdu.itslearning.com/plans/courses/50426/plan/407433?BackDestination=1#:~:text=udvekslings</v>
+      </c>
+      <c r="P72" t="str">
+        <v/>
+      </c>
+      <c r="Q72" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R72" t="str">
+        <v/>
+      </c>
+      <c r="S72" t="str">
+        <v/>
+      </c>
+      <c r="T72" t="str">
+        <v/>
+      </c>
+      <c r="U72" t="str">
+        <v/>
+      </c>
+      <c r="V72" t="str">
+        <v/>
+      </c>
+      <c r="W72" t="str">
+        <v/>
+      </c>
+      <c r="X72" t="str">
+        <v/>
+      </c>
+      <c r="Y72" t="str">
+        <v/>
+      </c>
+      <c r="Z72" t="str">
+        <v/>
+      </c>
+      <c r="AA72" t="str">
+        <v/>
+      </c>
+      <c r="AB72" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB72"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "foregår" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB72"/>
+  <dimension ref="A1:AB73"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6402,9 +6402,95 @@
         <v/>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>6758c1dc-05cd-42d9-b2c3-bbc31fa83971</v>
+      </c>
+      <c r="B73" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C73" t="str">
+        <v>foregår</v>
+      </c>
+      <c r="D73" t="str">
+        <v>foregå</v>
+      </c>
+      <c r="E73" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+      <c r="G73" t="str">
+        <v>-r, ..gik, -et</v>
+      </c>
+      <c r="H73" t="str">
+        <v>[ˈfɒːɒˌgɔˀ]</v>
+      </c>
+      <c r="I73" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014410_1.mp3</v>
+      </c>
+      <c r="J73" t="str">
+        <v>finde sted på et bestemt punkt i tid og sted eller på en bestemt måde om en begivenhed eller tidsbegrænset aktivitet</v>
+      </c>
+      <c r="K73" t="str">
+        <v>takes place</v>
+      </c>
+      <c r="L73" t="str">
+        <v>… formationsmøder, hvor du kan høre mere om dine muligheder, ansøgningsprocessen og få svar på dine spørgsmål. Der er både online og fysiske møder. Første møde er fysisk i Odense og foregår den 23/9. Du kan finde datoer og tilmeldingsmuligheder her: https://mitsdu.dk/en/mit_studie/bachelor/amerikanske_studier_bachelor/study_abroad/contact_and_guidance/information_mee …</v>
+      </c>
+      <c r="M73" t="str">
+        <v>Lecture 2 - Statistical Signal Processing, (E26) - itslearning</v>
+      </c>
+      <c r="N73" t="str">
+        <v>https://sdu.itslearning.com/plans/courses/50426/plan/407433?BackDestination=1</v>
+      </c>
+      <c r="O73" t="str">
+        <v>https://sdu.itslearning.com/plans/courses/50426/plan/407433?BackDestination=1#:~:text=foreg%C3%A5r</v>
+      </c>
+      <c r="P73" t="str">
+        <v/>
+      </c>
+      <c r="Q73" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R73" t="str">
+        <v/>
+      </c>
+      <c r="S73" t="str">
+        <v/>
+      </c>
+      <c r="T73" t="str">
+        <v/>
+      </c>
+      <c r="U73" t="str">
+        <v/>
+      </c>
+      <c r="V73" t="str">
+        <v/>
+      </c>
+      <c r="W73" t="str">
+        <v/>
+      </c>
+      <c r="X73" t="str">
+        <v/>
+      </c>
+      <c r="Y73" t="str">
+        <v/>
+      </c>
+      <c r="Z73" t="str">
+        <v/>
+      </c>
+      <c r="AA73" t="str">
+        <v/>
+      </c>
+      <c r="AB73" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB73"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "indsatsen" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB73"/>
+  <dimension ref="A1:AB74"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6488,9 +6488,95 @@
         <v/>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>19e4895b-d0e8-4c07-9c28-7e04b07968d0</v>
+      </c>
+      <c r="B74" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="C74" t="str">
+        <v>indsatsen</v>
+      </c>
+      <c r="D74" t="str">
+        <v>indsats</v>
+      </c>
+      <c r="E74" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F74" t="str">
+        <v>en</v>
+      </c>
+      <c r="G74" t="str">
+        <v>betydning 1-3: -en, -er, -erne</v>
+      </c>
+      <c r="H74" t="str">
+        <v>[ˈenˌsads]</v>
+      </c>
+      <c r="I74" t="str">
+        <v>https://static.ordnet.dk/mp3/11023/11023506_1.mp3</v>
+      </c>
+      <c r="J74" t="str">
+        <v>koncentreret virksomhed som man udøver for at opnå noget bestemt, fx for at løse et konkret problem, for at styrke et bestemt område eller for at vinde en sportskamp</v>
+      </c>
+      <c r="K74" t="str">
+        <v>The effort</v>
+      </c>
+      <c r="L74" t="str">
+        <v>Vil du have mulighed for at få ansvar for ESG-indsatsen hos vores nye samarbejdspartner? Vi søger lige nu en studerende, der har interesse for ESG og bæredygtighed, samt virksomhedens arbejde med data, rapportering og lovgivning.Hvem e …</v>
+      </c>
+      <c r="M74" t="str">
+        <v>Studiejob: ESG konsulent | JobTeaser</v>
+      </c>
+      <c r="N74" t="str">
+        <v>https://sdu.jobteaser.com/en/job-offers/b814dfc3-84f5-4f7c-a458-4a05c933f994-cand-studiejob-esg-konsulent</v>
+      </c>
+      <c r="O74" t="str">
+        <v>https://sdu.jobteaser.com/en/job-offers/b814dfc3-84f5-4f7c-a458-4a05c933f994-cand-studiejob-esg-konsulent#:~:text=indsatsen</v>
+      </c>
+      <c r="P74" t="str">
+        <v/>
+      </c>
+      <c r="Q74" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R74" t="str">
+        <v/>
+      </c>
+      <c r="S74" t="str">
+        <v/>
+      </c>
+      <c r="T74" t="str">
+        <v/>
+      </c>
+      <c r="U74" t="str">
+        <v/>
+      </c>
+      <c r="V74" t="str">
+        <v/>
+      </c>
+      <c r="W74" t="str">
+        <v/>
+      </c>
+      <c r="X74" t="str">
+        <v/>
+      </c>
+      <c r="Y74" t="str">
+        <v/>
+      </c>
+      <c r="Z74" t="str">
+        <v/>
+      </c>
+      <c r="AA74" t="str">
+        <v/>
+      </c>
+      <c r="AB74" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB74"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bæredygtighed" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB74"/>
+  <dimension ref="A1:AB75"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6574,9 +6574,95 @@
         <v/>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>7564e76c-d9e2-48c0-907f-1ebf6da55d1e</v>
+      </c>
+      <c r="B75" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="C75" t="str">
+        <v>bæredygtighed</v>
+      </c>
+      <c r="D75" t="str">
+        <v>bæredygtighed</v>
+      </c>
+      <c r="E75" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F75" t="str">
+        <v>en</v>
+      </c>
+      <c r="G75" t="str">
+        <v>-en</v>
+      </c>
+      <c r="H75" t="str">
+        <v>[ˈbεːʌˌdøgdiˌheðˀ]</v>
+      </c>
+      <c r="I75" t="str">
+        <v>https://static.ordnet.dk/mp3/51003/51003622_1.mp3</v>
+      </c>
+      <c r="J75" t="str">
+        <v>det at give et godt resultat der er i stand til at bestå over tid</v>
+      </c>
+      <c r="K75" t="str">
+        <v>Sustainability</v>
+      </c>
+      <c r="L75" t="str">
+        <v>Vil du have mulighed for at få ansvar for ESG-indsatsen hos vores nye samarbejdspartner? Vi søger lige nu en studerende, der har interesse for ESG og bæredygtighed, samt virksomhedens arbejde med data, rapportering og lovgivning.Hvem er Cand?Cand skaber udviklingsmuligheder i samspillet mellem studerende og virksomheder. Vi gør det nemt for …</v>
+      </c>
+      <c r="M75" t="str">
+        <v>Studiejob: ESG konsulent | JobTeaser</v>
+      </c>
+      <c r="N75" t="str">
+        <v>https://sdu.jobteaser.com/en/job-offers/b814dfc3-84f5-4f7c-a458-4a05c933f994-cand-studiejob-esg-konsulent</v>
+      </c>
+      <c r="O75" t="str">
+        <v>https://sdu.jobteaser.com/en/job-offers/b814dfc3-84f5-4f7c-a458-4a05c933f994-cand-studiejob-esg-konsulent#:~:text=b%C3%A6redygtighed</v>
+      </c>
+      <c r="P75" t="str">
+        <v/>
+      </c>
+      <c r="Q75" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R75" t="str">
+        <v/>
+      </c>
+      <c r="S75" t="str">
+        <v/>
+      </c>
+      <c r="T75" t="str">
+        <v/>
+      </c>
+      <c r="U75" t="str">
+        <v/>
+      </c>
+      <c r="V75" t="str">
+        <v/>
+      </c>
+      <c r="W75" t="str">
+        <v/>
+      </c>
+      <c r="X75" t="str">
+        <v/>
+      </c>
+      <c r="Y75" t="str">
+        <v/>
+      </c>
+      <c r="Z75" t="str">
+        <v/>
+      </c>
+      <c r="AA75" t="str">
+        <v/>
+      </c>
+      <c r="AB75" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB75"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Afdeling" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB75"/>
+  <dimension ref="A1:AB76"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6660,9 +6660,95 @@
         <v/>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>617fdad5-c6db-4dd6-b2bb-dae374648c75</v>
+      </c>
+      <c r="B76" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Afdeling</v>
+      </c>
+      <c r="D76" t="str">
+        <v>afdeling</v>
+      </c>
+      <c r="E76" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F76" t="str">
+        <v>en</v>
+      </c>
+      <c r="G76" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H76" t="str">
+        <v>[ˈɑwˌdeˀleŋ]</v>
+      </c>
+      <c r="I76" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000325_1.mp3</v>
+      </c>
+      <c r="J76" t="str">
+        <v>organisatorisk del af et større hele fx et hospital, en bank, en virksomhed, en forening, en hær eller en offentlig myndighed</v>
+      </c>
+      <c r="K76" t="str">
+        <v>Department</v>
+      </c>
+      <c r="L76" t="str">
+        <v>Afdeling Fraugde-Kærby</v>
+      </c>
+      <c r="M76" t="str">
+        <v>Find Os | Rosa Danica</v>
+      </c>
+      <c r="N76" t="str">
+        <v>https://www.rosa-danica.dk/find-us/</v>
+      </c>
+      <c r="O76" t="str">
+        <v>https://www.rosa-danica.dk/find-us/#:~:text=Afdeling</v>
+      </c>
+      <c r="P76" t="str">
+        <v/>
+      </c>
+      <c r="Q76" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R76" t="str">
+        <v/>
+      </c>
+      <c r="S76" t="str">
+        <v/>
+      </c>
+      <c r="T76" t="str">
+        <v/>
+      </c>
+      <c r="U76" t="str">
+        <v/>
+      </c>
+      <c r="V76" t="str">
+        <v/>
+      </c>
+      <c r="W76" t="str">
+        <v/>
+      </c>
+      <c r="X76" t="str">
+        <v/>
+      </c>
+      <c r="Y76" t="str">
+        <v/>
+      </c>
+      <c r="Z76" t="str">
+        <v/>
+      </c>
+      <c r="AA76" t="str">
+        <v/>
+      </c>
+      <c r="AB76" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB76"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "skyde" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB76"/>
+  <dimension ref="A1:AB77"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6746,9 +6746,95 @@
         <v/>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>88e4bba9-221e-4bc5-a706-c97f77671631</v>
+      </c>
+      <c r="B77" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="C77" t="str">
+        <v>skyde</v>
+      </c>
+      <c r="D77" t="str">
+        <v>skyde</v>
+      </c>
+      <c r="E77" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+      <c r="G77" t="str">
+        <v>-r, skød, skudt</v>
+      </c>
+      <c r="H77" t="str">
+        <v>[ˈsgyːðə]</v>
+      </c>
+      <c r="I77" t="str">
+        <v>https://static.ordnet.dk/mp3/11047/11047251_1.mp3</v>
+      </c>
+      <c r="J77" t="str">
+        <v>affyre et skud med et skydevåben</v>
+      </c>
+      <c r="K77" t="str">
+        <v>shoot</v>
+      </c>
+      <c r="L77" t="str">
+        <v>Kampfly styrtede tirsdag ned nær den amerikanske Spangdahlem-luftbase i det vestlige Tyskland. Piloten overlevede ved at skyde sig ud med katapultsædet, mens én person på jorden blev såret.</v>
+      </c>
+      <c r="M77" t="str">
+        <v>Pilot hoppede ud med katapult: Amerikansk F-16-kampfly styrter ned i Tyskland | Ingeniøren</v>
+      </c>
+      <c r="N77" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O77" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=skyde</v>
+      </c>
+      <c r="P77" t="str">
+        <v/>
+      </c>
+      <c r="Q77" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R77" t="str">
+        <v/>
+      </c>
+      <c r="S77" t="str">
+        <v/>
+      </c>
+      <c r="T77" t="str">
+        <v/>
+      </c>
+      <c r="U77" t="str">
+        <v/>
+      </c>
+      <c r="V77" t="str">
+        <v/>
+      </c>
+      <c r="W77" t="str">
+        <v/>
+      </c>
+      <c r="X77" t="str">
+        <v/>
+      </c>
+      <c r="Y77" t="str">
+        <v/>
+      </c>
+      <c r="Z77" t="str">
+        <v/>
+      </c>
+      <c r="AA77" t="str">
+        <v/>
+      </c>
+      <c r="AB77" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB77"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "anerkendt" to Random.xlsx
</commit_message>
<xml_diff>
--- a/sets/Random.xlsx
+++ b/sets/Random.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB77"/>
+  <dimension ref="A1:AB78"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6832,9 +6832,95 @@
         <v/>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>9730c044-4724-477a-8a9d-b1f7dd00f057</v>
+      </c>
+      <c r="B78" t="str">
+        <v>2026-10-12</v>
+      </c>
+      <c r="C78" t="str">
+        <v>anerkendt</v>
+      </c>
+      <c r="D78" t="str">
+        <v>anerkende</v>
+      </c>
+      <c r="E78" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+      <c r="G78" t="str">
+        <v>-r, ..kendte, ..kendt</v>
+      </c>
+      <c r="H78" t="str">
+        <v>[ˈanʌˌkεnˀə]</v>
+      </c>
+      <c r="I78" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001739_1.mp3</v>
+      </c>
+      <c r="J78" t="str">
+        <v>erkende som sandt eller berettiget</v>
+      </c>
+      <c r="K78" t="str">
+        <v>Recognized</v>
+      </c>
+      <c r="L78" t="str">
+        <v>Lurpak® er globalt anerkendt for enestående kvalitet og smag. Et ry, der er opbygget og fortsat styrkes, gennem hårdt arbejde, dedikation og sans for detaljen.</v>
+      </c>
+      <c r="M78" t="str">
+        <v>Vi fejrer 125 år med Lurpak® | Lurpak®</v>
+      </c>
+      <c r="N78" t="str">
+        <v>https://www.lurpak.com/da/vores-historie/?utm_source=fbig&amp;utm_medium=paid&amp;utm_campaign=26_dk_lurp_125anniversary_41_44_reach%3A3300101308_organic-boost&amp;utm_content=dk_lurp_125anniversary_price_vid31+_4x5_fbig_da_b9cc60&amp;utm_id=120251060710430429&amp;utm_term=120251060727290429&amp;fbclid=IwY2xjawU5nsVleHRuA2FlbQEwAHBkb2YBYWRpZAGrN7PgWKhdYnJpZBEwdHp1cVJLdXJrc2w1TmM5RHNydGMGYXBwX2lkEDIyMjAzOTE3ODgyMDA4OTIAAR6hSFwEorfWq7-fUHZs_z1s1ydyprPUuSau1MqxfsNJ6bRdVTiwkCUvyrEv5A_aem_l9OGtSb8-zhk4MsUGbViIA&amp;campaign_id=120251060710430429&amp;ad_id=120251060727320429</v>
+      </c>
+      <c r="O78" t="str">
+        <v>https://www.lurpak.com/da/vores-historie/?utm_source=fbig&amp;utm_medium=paid&amp;utm_campaign=26_dk_lurp_125anniversary_41_44_reach%3A3300101308_organic-boost&amp;utm_content=dk_lurp_125anniversary_price_vid31+_4x5_fbig_da_b9cc60&amp;utm_id=120251060710430429&amp;utm_term=120251060727290429&amp;fbclid=IwY2xjawU5nsVleHRuA2FlbQEwAHBkb2YBYWRpZAGrN7PgWKhdYnJpZBEwdHp1cVJLdXJrc2w1TmM5RHNydGMGYXBwX2lkEDIyMjAzOTE3ODgyMDA4OTIAAR6hSFwEorfWq7-fUHZs_z1s1ydyprPUuSau1MqxfsNJ6bRdVTiwkCUvyrEv5A_aem_l9OGtSb8-zhk4MsUGbViIA&amp;campaign_id=120251060710430429&amp;ad_id=120251060727320429#:~:text=anerkendt</v>
+      </c>
+      <c r="P78" t="str">
+        <v/>
+      </c>
+      <c r="Q78" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R78" t="str">
+        <v/>
+      </c>
+      <c r="S78" t="str">
+        <v/>
+      </c>
+      <c r="T78" t="str">
+        <v/>
+      </c>
+      <c r="U78" t="str">
+        <v/>
+      </c>
+      <c r="V78" t="str">
+        <v/>
+      </c>
+      <c r="W78" t="str">
+        <v/>
+      </c>
+      <c r="X78" t="str">
+        <v/>
+      </c>
+      <c r="Y78" t="str">
+        <v/>
+      </c>
+      <c r="Z78" t="str">
+        <v/>
+      </c>
+      <c r="AA78" t="str">
+        <v/>
+      </c>
+      <c r="AB78" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB78"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>